<commit_message>
feat(tool:arch): add solution reports and drawio export
</commit_message>
<xml_diff>
--- a/tests/otdev/fixtures/arch/architecture.xlsx
+++ b/tests/otdev/fixtures/arch/architecture.xlsx
@@ -10,8 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sys" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="app" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cmp" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="int" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="interface" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="usr" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="project" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="project_scope" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -686,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -702,15 +704,20 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>src</t>
+          <t>provider</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>dst</t>
+          <t>consumer</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
+        <is>
+          <t>interaction_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
@@ -719,7 +726,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>int_auth_ui</t>
+          <t>interface_auth_ui</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -729,15 +736,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>cmp_ui</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>cmp_auth</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>cmp_ui</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>core</t>
         </is>
@@ -746,7 +758,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>int_user_api</t>
+          <t>interface_user_api</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -756,15 +768,180 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>app_api</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>usr_ops</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>interface_core_legacy</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Core to Legacy Batch</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>sys_core</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>sys_legacy</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>interface_ui_worker</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>UI to Worker Queue</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cmp_ui</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>cmp_old</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>queue</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>interface_api_worker</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>API to Worker File</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>app_api</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>cmp_old</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>interface_admin_worker</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Admin to Worker Pubsub</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>app_admin</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>app_old</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>pubsub</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>interface_auth_worker</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Auth to Worker API</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>cmp_auth</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>cmp_old</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>api</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>core</t>
         </is>
@@ -831,4 +1008,484 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>detail_level</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>connect_level</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Wallet Project</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>wip</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>item_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>item_id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>change_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>sys_core</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>application</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>app_api</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>cmp_old</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>interface</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>interface_core_legacy</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>dependency</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>interface</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>interface_user_api</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>changed</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>application</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>app_admin</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>impacted</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>sys_core</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>impacted</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>cmp_auth</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>